<commit_message>
wip before it touch the fertility startup script
</commit_message>
<xml_diff>
--- a/ProsperPerishCalcs/analysis/building_levels/data/goods_output_modifiers.xlsx
+++ b/ProsperPerishCalcs/analysis/building_levels/data/goods_output_modifiers.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Info" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RGO" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,11 +418,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>good</t>
-        </is>
-      </c>
       <c r="B1" t="inlineStr">
         <is>
           <t>flatland</t>
@@ -686,7 +681,7 @@
         <v>0.05</v>
       </c>
       <c r="R3" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
         <v>-0.35</v>
@@ -792,7 +787,7 @@
         <v>0.05</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5">
@@ -874,7 +869,7 @@
         <v>0.1</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="6">
@@ -956,7 +951,7 @@
         <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="7">
@@ -1038,7 +1033,7 @@
         <v>0.08</v>
       </c>
       <c r="Z7" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="8">
@@ -1120,7 +1115,7 @@
         <v>0.08</v>
       </c>
       <c r="Z8" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="9">
@@ -1284,7 +1279,7 @@
         <v>0.1</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="11">
@@ -1366,7 +1361,7 @@
         <v>0.05</v>
       </c>
       <c r="Z11" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="12">
@@ -1458,76 +1453,76 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>-0.35</v>
+        <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
@@ -1708,29 +1703,623 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>good_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>output_modifier</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>peasants_food</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Per-cell bounds: [-0.35, 0.35]</t>
-        </is>
+          <t>beeswax</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-0.025</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sum across applicable attributes. Values clamped and rounded to 2 decimals.</t>
-        </is>
-      </c>
+          <t>chili</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cloves</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cocoa</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>coffee</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cotton</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dyes</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>elephants</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fiber_crops</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>horses</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>incense</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>legumes</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>livestock</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>maize</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>millet</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>olives</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>pepper</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>potato</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>rice</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>saffron</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>silk</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sugar</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>tea</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>tobacco</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>wheat</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>wine</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>wool</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>lumber</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>amber</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>clay</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fish</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>medicaments</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>pearls</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>salt</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>sand</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fur</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ivory</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>wild_game</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>-0.035</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>alum</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>coal</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>gems</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>goods_gold</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>lead</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>marble</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>mercury</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>saltpeter</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>silver</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>stone</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>tin</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>